<commit_message>
feat(popup): land handoff 03 - pilot fixes F1-F6, -002-05 generated, 5 TCs green
- apply R-POP15 F1-F6 to all pilot TCs (check targets, quoting, drop
  environment preconditions, input_test_data=NA, rewrite -002-02 reasoning
  to R-POP12's ground)
- renumber TC IDs to NR1L-Popup-001..005 per R-POP13
- generate -002-05 from the GP4-4 requirement text, no PU cited (R-POP14)
- lint_docs036: in-table duplicates stay red, cross-table downgraded to
  note, prefix extraction limited to the leading table, explicit
  "no series detected" on blind spots (R-POP16)
- add scripts/ledger_xref.py: package/ruling references cross-checked
  against the feature ledger (R-POP17); fixes two live popup defects
- log verified numbering gaps to audio_mgmt and time_management BACKLOG
- register A-POP10 (leading-table criterion loses true positives) and
  A-POP11 (sxm entries were false positives, not amended)
- regenerate RULINGS.sha.tsv: +6 rows, no existing sha changed
</commit_message>
<xml_diff>
--- a/features/popup/sandbox/pilot01/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_20260817_ext.xlsx
+++ b/features/popup/sandbox/pilot01/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_20260817_ext.xlsx
@@ -7897,7 +7897,7 @@
       <c r="E10" s="81"/>
       <c r="F10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">newR1L-POP-001</t>
+          <t xml:space="preserve">NR1L-Popup-001</t>
         </is>
       </c>
       <c r="G10" s="81" t="inlineStr">
@@ -7918,25 +7918,24 @@
       </c>
       <c r="J10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The vehicle is stationary with the ignition in RUN
-2. The Home Screen is displayed</t>
+          <t xml:space="preserve">1. The Home Screen is displayed</t>
         </is>
       </c>
       <c r="K10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time-out = 5 s, as defined by PU0942 Timeout (sec)</t>
+          <t xml:space="preserve">NA</t>
         </is>
       </c>
       <c r="L10" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Enter the Home Screen page-management view and add a home screen page
 2. Leave the screen and all buttons untouched for 10 seconds after the pop-up appears
-3. Read the pop-up display status and the elapsed time at the moment the pop-up disappears</t>
+3. Read the pop-up display status and the elapsed time and check that the pop-up has closed by itself 5 seconds after it appeared, matching the Time-out defined by PU0942 Timeout (sec)</t>
         </is>
       </c>
       <c r="M10" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The pop-up is displayed showing `&lt;X&gt;` and `Page added! [Reorder]`, as defined by PU0942 String/Popup Message
+          <t xml:space="preserve">1. The pop-up is displayed showing "&lt;X&gt;" and "Page added! [Reorder]", as defined by PU0942 String/Popup Message
 2. No user interaction is registered during the 10-second window
 3. The pop-up closes by itself 5 seconds after it appeared, matching the Time-out defined by PU0942 Timeout (sec), and the Home Screen is shown without the pop-up</t>
         </is>
@@ -8002,7 +8001,7 @@
       <c r="E11" s="81"/>
       <c r="F11" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">newR1L-POP-002</t>
+          <t xml:space="preserve">NR1L-Popup-002</t>
         </is>
       </c>
       <c r="G11" s="81" t="inlineStr">
@@ -8018,14 +8017,13 @@
       <c r="I11" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">Pop-ups can be closed after pressing button that opened pop-up again (eg. Tracks popups)
-(Second press of the opening control `&lt;Trks&gt;`, PU0215)</t>
+(Second press of the opening control &lt;Trks&gt;, PU0215)</t>
         </is>
       </c>
       <c r="J11" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The vehicle is stationary with the ignition in RUN
-2. A media source containing at least one track list is available
-3. The Media screen is displayed</t>
+          <t xml:space="preserve">1. A media source containing at least one track list is available
+2. The Media screen is displayed</t>
         </is>
       </c>
       <c r="K11" s="81" t="inlineStr">
@@ -8035,15 +8033,15 @@
       </c>
       <c r="L11" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. On the Media screen, press the Track list button `&lt;Trks&gt;`
-2. Press `&lt;Trks&gt;` a second time while the pop-up is displayed
-3. Read the pop-up display status immediately after the second press</t>
+          <t xml:space="preserve">1. On the Media screen, press the Track list button "Trks"
+2. Press "Trks" a second time while the pop-up is displayed
+3. Read the pop-up display status immediately after the second press and check that the pop-up is no longer displayed</t>
         </is>
       </c>
       <c r="M11" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The `Tracks List` pop-up is displayed, as defined by PU0215 String/Popup Message
-2. The second press lands on the same `&lt;Trks&gt;` button that opened the pop-up
+          <t xml:space="preserve">1. The "Tracks List" pop-up is displayed, as defined by PU0215 String/Popup Message
+2. The second press lands on the same "&lt;Trks&gt;" button that opened the pop-up
 3. The pop-up is closed and the Media screen is shown without the pop-up</t>
         </is>
       </c>
@@ -8109,7 +8107,7 @@
       <c r="E12" s="81"/>
       <c r="F12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">newR1L-POP-003</t>
+          <t xml:space="preserve">NR1L-Popup-003</t>
         </is>
       </c>
       <c r="G12" s="81" t="inlineStr">
@@ -8130,26 +8128,25 @@
       </c>
       <c r="J12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The vehicle is stationary with the ignition in RUN
-2. At least two driver Profiles exist on the head unit
-3. The All Profiles tab is reachable from the current screen</t>
+          <t xml:space="preserve">1. At least two driver Profiles exist on the head unit
+2. The All Profiles tab is reachable from the current screen</t>
         </is>
       </c>
       <c r="K12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time-out = 5 s, as defined by PU0580 Timeout (sec)</t>
+          <t xml:space="preserve">NA</t>
         </is>
       </c>
       <c r="L12" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Open the All Profiles tab and switch manually to another Profile
 2. Within 5 seconds of the pop-up appearing, tap an area of the screen outside the pop-up window frame
-3. Read the pop-up display status immediately after the tap</t>
+3. Read the pop-up display status immediately after the tap and check that the pop-up is no longer displayed, before the 5-second Time-out defined by PU0580 Timeout (sec) has elapsed</t>
         </is>
       </c>
       <c r="M12" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The pop-up is displayed showing `"Welcome [username]", "X"`, as defined by PU0580 String/Popup Message
+          <t xml:space="preserve">1. The pop-up is displayed showing "Welcome [username]", "X", as defined by PU0580 String/Popup Message
 2. The tap lands outside the pop-up window frame and activates no pop-up control
 3. The pop-up is closed, and the closure occurs before the 5-second Time-out defined by PU0580 Timeout (sec) elapses</t>
         </is>
@@ -8215,7 +8212,7 @@
       <c r="E13" s="81"/>
       <c r="F13" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">newR1L-POP-004</t>
+          <t xml:space="preserve">NR1L-Popup-004</t>
         </is>
       </c>
       <c r="G13" s="81" t="inlineStr">
@@ -8231,32 +8228,31 @@
       <c r="I13" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">Pop-ups can be closed after making a selection inside the pop-up if applicable
-(Selection `&lt;OK&gt;` inside the pop-up, PU0949)</t>
+(Selection &lt;OK&gt; inside the pop-up, PU0949)</t>
         </is>
       </c>
       <c r="J13" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The vehicle is stationary with the ignition in RUN
-2. No mobile phone is paired with the head unit
-3. The Home Screen Shortcuts view is displayed</t>
+          <t xml:space="preserve">1. No mobile phone is paired with the head unit
+2. The Home Screen Shortcuts view is displayed</t>
         </is>
       </c>
       <c r="K13" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Time-out = 3 s, as defined by PU0949 Timeout (sec)</t>
+          <t xml:space="preserve">NA</t>
         </is>
       </c>
       <c r="L13" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">1. On the Home Screen Shortcuts view, press the grayed out "Make a Call" button
-2. Within 3 seconds of the pop-up appearing, press `&lt;OK&gt;` inside the pop-up
-3. Read the pop-up display status immediately after the press</t>
+2. Within 3 seconds of the pop-up appearing, press "OK" inside the pop-up
+3. Read the pop-up display status immediately after the press and check that the pop-up is no longer displayed, before the 3-second Time-out defined by PU0949 Timeout (sec) has elapsed</t>
         </is>
       </c>
       <c r="M13" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The pop-up is displayed showing `No Phone is Connected.        &lt;OK&gt;    &lt;X&gt;`, as defined by PU0949 String/Popup Message
-2. The `&lt;OK&gt;` press is registered while the pop-up is still displayed
+          <t xml:space="preserve">1. The pop-up is displayed showing "No Phone is Connected.        &lt;OK&gt;    &lt;X&gt;", as defined by PU0949 String/Popup Message
+2. The "&lt;OK&gt;" press is registered while the pop-up is still displayed
 3. The pop-up is closed, and the closure occurs before the 3-second Time-out defined by PU0949 Timeout (sec) elapses</t>
         </is>
       </c>
@@ -8313,22 +8309,84 @@
         <v/>
       </c>
       <c r="C14" s="82"/>
-      <c r="D14" s="81"/>
+      <c r="D14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SWE1-POP-002-05</t>
+        </is>
+      </c>
       <c r="E14" s="81"/>
-      <c r="F14" s="81"/>
-      <c r="G14" s="81"/>
-      <c r="H14" s="81"/>
-      <c r="I14" s="81"/>
-      <c r="J14" s="81"/>
-      <c r="K14" s="81"/>
-      <c r="L14" s="81"/>
-      <c r="M14" s="81"/>
-      <c r="N14" s="81"/>
-      <c r="O14" s="81"/>
-      <c r="P14" s="81"/>
+      <c r="F14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NR1L-Popup-005</t>
+        </is>
+      </c>
+      <c r="G14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Popup</t>
+        </is>
+      </c>
+      <c r="H14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pop-up Close</t>
+        </is>
+      </c>
+      <c r="I14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exceptions when the popup allows the user to perform more than 1 task- e.g in the search keyboard only X button 'close', any other buttons do not close the popup
+(Non-closing control inside a multi-task pop-up; no PU cited)</t>
+        </is>
+      </c>
+      <c r="J14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. A pop-up that allows the user to perform more than 1 task is available, the search keyboard being the example given in the requirement
+2. That pop-up is displayed</t>
+        </is>
+      </c>
+      <c r="K14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
+      <c r="L14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Trigger the pop-up that allows the user to perform more than 1 task
+2. Inside the displayed pop-up, press a button other than the "X" button
+3. Read the pop-up display status immediately after the press and check that the pop-up is still displayed</t>
+        </is>
+      </c>
+      <c r="M14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. The pop-up is displayed and allows the user to perform more than 1 task
+2. The button pressed is a button other than the "X" button of that pop-up
+3. The pop-up is not closed by that press and remains displayed</t>
+        </is>
+      </c>
+      <c r="N14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYS1_HMI_Core_HMI_Logic_and_Flow_R1_SR24_Post_2A_(February_2_2023)_5.6</t>
+        </is>
+      </c>
+      <c r="O14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NEW</t>
+        </is>
+      </c>
+      <c r="P14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
       <c r="Q14" s="81"/>
-      <c r="R14" s="81"/>
-      <c r="S14" s="81"/>
+      <c r="R14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">狀態轉換 (State Transition Testing)</t>
+        </is>
+      </c>
+      <c r="S14" s="81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NA</t>
+        </is>
+      </c>
       <c r="T14" s="81"/>
       <c r="U14" s="81"/>
       <c r="V14" s="81"/>
@@ -8336,7 +8394,11 @@
       <c r="X14" s="83"/>
       <c r="Y14" s="81"/>
       <c r="Z14" s="83"/>
-      <c r="AA14" s="83"/>
+      <c r="AA14" s="83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PeiPYHsu</t>
+        </is>
+      </c>
       <c r="AB14" s="81"/>
       <c r="AC14" s="81"/>
       <c r="AD14" s="81"/>

</xml_diff>